<commit_message>
Se agrega 1 persona al registro
</commit_message>
<xml_diff>
--- a/backend/Personal MINEDUCYT.xlsx
+++ b/backend/Personal MINEDUCYT.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Recuperacion\Documents\SOLICITUD TRANSPORTE\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Recuperacion\Documents\sistema-transporte\backend\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B5316284-DEFB-4789-8DD5-D823754EB09A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DBF16AC-2B88-4322-AD34-AB04BC04C0F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-4815" windowWidth="29040" windowHeight="15990" xr2:uid="{2FACA3CF-F98D-4E51-8367-D061FBCF9444}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11310" xr2:uid="{2FACA3CF-F98D-4E51-8367-D061FBCF9444}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="19">
   <si>
     <t>Motoristas</t>
   </si>
@@ -93,6 +93,9 @@
   </si>
   <si>
     <t>Alexis Paniagua</t>
+  </si>
+  <si>
+    <t>Mauricio Escobar</t>
   </si>
 </sst>
 </file>
@@ -148,8 +151,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{08EBA544-43DC-474C-AB2C-A10F7DDEA4FC}" name="Tabla2" displayName="Tabla2" ref="A1:B17" totalsRowShown="0">
-  <autoFilter ref="A1:B17" xr:uid="{08EBA544-43DC-474C-AB2C-A10F7DDEA4FC}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{08EBA544-43DC-474C-AB2C-A10F7DDEA4FC}" name="Tabla2" displayName="Tabla2" ref="A1:B18" totalsRowShown="0">
+  <autoFilter ref="A1:B18" xr:uid="{08EBA544-43DC-474C-AB2C-A10F7DDEA4FC}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{25771EF2-CE0F-4965-9543-DE434F865257}" name="Motoristas"/>
     <tableColumn id="2" xr3:uid="{74C532D8-30C6-43D4-9961-4055539A669C}" name="Personal"/>
@@ -475,7 +478,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{067AF64D-7B65-4F81-8CDE-D8C18B07C4E4}">
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.5703125" customWidth="1"/>
@@ -539,6 +542,9 @@
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>18</v>
+      </c>
       <c r="B8" t="s">
         <v>17</v>
       </c>
@@ -586,6 +592,11 @@
     <row r="17" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
         <v>11</v>
+      </c>
+    </row>
+    <row r="18" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B18" t="s">
+        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Se agrega a Miguel
</commit_message>
<xml_diff>
--- a/backend/Personal MINEDUCYT.xlsx
+++ b/backend/Personal MINEDUCYT.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Recuperacion\Documents\sistema-transporte\backend\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EAC3E87E-D694-46FE-85D0-46F411B250F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02A47413-1503-4780-938D-79924DBF092B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11310" xr2:uid="{2FACA3CF-F98D-4E51-8367-D061FBCF9444}"/>
+    <workbookView xWindow="1860" yWindow="1860" windowWidth="15375" windowHeight="7995" xr2:uid="{2FACA3CF-F98D-4E51-8367-D061FBCF9444}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -92,13 +92,13 @@
     <t>Cintia Sandoval</t>
   </si>
   <si>
-    <t>Guadalupe Franco</t>
-  </si>
-  <si>
     <t>Heidi Arana</t>
   </si>
   <si>
     <t>Erika Linares</t>
+  </si>
+  <si>
+    <t>Miguel Izquierdo</t>
   </si>
 </sst>
 </file>
@@ -526,7 +526,7 @@
         <v>4</v>
       </c>
       <c r="B4" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -555,7 +555,7 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
@@ -566,7 +566,7 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Cambio de plantilla y reconfiguración de frontend.
</commit_message>
<xml_diff>
--- a/backend/Personal MINEDUCYT.xlsx
+++ b/backend/Personal MINEDUCYT.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Recuperacion\Documents\sistema-transporte\backend\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C681FC25-EAC2-44CF-863F-D5AE74C0F85A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B12B6B0A-8732-47F1-8514-385D1DF26344}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11310" xr2:uid="{2FACA3CF-F98D-4E51-8367-D061FBCF9444}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="39">
   <si>
     <t>Motoristas</t>
   </si>
@@ -99,6 +99,63 @@
   </si>
   <si>
     <t>Miguel Izquierdo</t>
+  </si>
+  <si>
+    <t>7438-4652</t>
+  </si>
+  <si>
+    <t>6070-6616</t>
+  </si>
+  <si>
+    <t>6420-5959</t>
+  </si>
+  <si>
+    <t>7839-3152</t>
+  </si>
+  <si>
+    <t>7488-3301</t>
+  </si>
+  <si>
+    <t>7251-7471</t>
+  </si>
+  <si>
+    <t>7892-8974</t>
+  </si>
+  <si>
+    <t>6861-5338</t>
+  </si>
+  <si>
+    <t>6061-2421</t>
+  </si>
+  <si>
+    <t>7860-2484</t>
+  </si>
+  <si>
+    <t>7961-3643</t>
+  </si>
+  <si>
+    <t>6027-9205</t>
+  </si>
+  <si>
+    <t>7495-9192</t>
+  </si>
+  <si>
+    <t>7874-2819</t>
+  </si>
+  <si>
+    <t>7899-7973</t>
+  </si>
+  <si>
+    <t>7200-8336</t>
+  </si>
+  <si>
+    <t>7070-9667</t>
+  </si>
+  <si>
+    <t>7070-9518</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Teléfono </t>
   </si>
 </sst>
 </file>
@@ -163,11 +220,12 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{08EBA544-43DC-474C-AB2C-A10F7DDEA4FC}" name="Tabla2" displayName="Tabla2" ref="A1:B19" totalsRowShown="0">
-  <autoFilter ref="A1:B19" xr:uid="{08EBA544-43DC-474C-AB2C-A10F7DDEA4FC}"/>
-  <tableColumns count="2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{08EBA544-43DC-474C-AB2C-A10F7DDEA4FC}" name="Tabla2" displayName="Tabla2" ref="A1:C19" totalsRowShown="0">
+  <autoFilter ref="A1:C19" xr:uid="{08EBA544-43DC-474C-AB2C-A10F7DDEA4FC}"/>
+  <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{25771EF2-CE0F-4965-9543-DE434F865257}" name="Motoristas"/>
     <tableColumn id="2" xr3:uid="{74C532D8-30C6-43D4-9961-4055539A669C}" name="Personal"/>
+    <tableColumn id="3" xr3:uid="{DF47E11E-4B1F-4787-9050-3139BCD1D5CD}" name="Teléfono "/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -504,6 +562,9 @@
       <c r="B1" t="s">
         <v>1</v>
       </c>
+      <c r="C1" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
@@ -512,6 +573,9 @@
       <c r="B2" t="s">
         <v>5</v>
       </c>
+      <c r="C2" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
@@ -520,6 +584,9 @@
       <c r="B3" t="s">
         <v>6</v>
       </c>
+      <c r="C3" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
@@ -528,6 +595,9 @@
       <c r="B4" t="s">
         <v>19</v>
       </c>
+      <c r="C4" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
@@ -536,6 +606,9 @@
       <c r="B5" t="s">
         <v>16</v>
       </c>
+      <c r="C5" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
@@ -544,6 +617,9 @@
       <c r="B6" t="s">
         <v>11</v>
       </c>
+      <c r="C6" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
@@ -552,6 +628,9 @@
       <c r="B7" t="s">
         <v>12</v>
       </c>
+      <c r="C7" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
@@ -560,61 +639,97 @@
       <c r="B8" t="s">
         <v>18</v>
       </c>
+      <c r="C8" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
         <v>8</v>
       </c>
+      <c r="C9" t="s">
+        <v>27</v>
+      </c>
       <c r="F9" s="1"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>17</v>
       </c>
+      <c r="C10" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
         <v>10</v>
       </c>
+      <c r="C11" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
         <v>2</v>
       </c>
+      <c r="C12" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
         <v>15</v>
       </c>
+      <c r="C13" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
         <v>3</v>
       </c>
+      <c r="C14" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
         <v>4</v>
       </c>
+      <c r="C15" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="17" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C16" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="17" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="18" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C17" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="18" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="19" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C18" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="19" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B19" t="s">
         <v>9</v>
+      </c>
+      <c r="C19" t="s">
+        <v>37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>